<commit_message>
Keep Russian as translation language
</commit_message>
<xml_diff>
--- a/data/source/Saved translations.xlsx
+++ b/data/source/Saved translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saved translations" sheetId="1" r:id="Rc2220abad3a94c84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saved translations" sheetId="1" r:id="R8eadaa960bcf4be1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3902,16 +3902,16 @@
     </x:row>
     <x:row r="262">
       <x:c r="A262" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B262" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C262" s="1" t="str">
+        <x:v>pitfalls</x:v>
+      </x:c>
+      <x:c r="D262" s="1" t="str">
         <x:v>подводные камни</x:v>
-      </x:c>
-      <x:c r="D262" s="1" t="str">
-        <x:v>pitfalls</x:v>
       </x:c>
     </x:row>
     <x:row r="263">
@@ -4126,30 +4126,30 @@
     </x:row>
     <x:row r="278">
       <x:c r="A278" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B278" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C278" s="1" t="str">
+        <x:v>On horseback</x:v>
+      </x:c>
+      <x:c r="D278" s="1" t="str">
         <x:v>Фверзом на лошали</x:v>
-      </x:c>
-      <x:c r="D278" s="1" t="str">
-        <x:v>On horseback</x:v>
       </x:c>
     </x:row>
     <x:row r="279">
       <x:c r="A279" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B279" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C279" s="1" t="str">
+        <x:v>imprint of war</x:v>
+      </x:c>
+      <x:c r="D279" s="1" t="str">
         <x:v>отпечаток войны</x:v>
-      </x:c>
-      <x:c r="D279" s="1" t="str">
-        <x:v>imprint of war</x:v>
       </x:c>
     </x:row>
     <x:row r="280">
@@ -5750,16 +5750,16 @@
     </x:row>
     <x:row r="394">
       <x:c r="A394" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B394" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C394" s="1" t="str">
+        <x:v>Garnish</x:v>
+      </x:c>
+      <x:c r="D394" s="1" t="str">
         <x:v>Гарнир</x:v>
-      </x:c>
-      <x:c r="D394" s="1" t="str">
-        <x:v>Garnish</x:v>
       </x:c>
     </x:row>
     <x:row r="395">
@@ -6212,16 +6212,16 @@
     </x:row>
     <x:row r="427">
       <x:c r="A427" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B427" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C427" s="1" t="str">
+        <x:v>Okay, let's say</x:v>
+      </x:c>
+      <x:c r="D427" s="1" t="str">
         <x:v>Хорошо, допустим</x:v>
-      </x:c>
-      <x:c r="D427" s="1" t="str">
-        <x:v>Okay, let's say</x:v>
       </x:c>
     </x:row>
     <x:row r="428">
@@ -6688,16 +6688,16 @@
     </x:row>
     <x:row r="461">
       <x:c r="A461" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B461" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C461" s="1" t="str">
+        <x:v>virginity</x:v>
+      </x:c>
+      <x:c r="D461" s="1" t="str">
         <x:v>девственность</x:v>
-      </x:c>
-      <x:c r="D461" s="1" t="str">
-        <x:v>virginity</x:v>
       </x:c>
     </x:row>
     <x:row r="462">
@@ -6800,16 +6800,16 @@
     </x:row>
     <x:row r="469">
       <x:c r="A469" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B469" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C469" s="1" t="str">
+        <x:v>conclusion, inference</x:v>
+      </x:c>
+      <x:c r="D469" s="1" t="str">
         <x:v>вывод, умозаключение</x:v>
-      </x:c>
-      <x:c r="D469" s="1" t="str">
-        <x:v>conclusion, inference</x:v>
       </x:c>
     </x:row>
     <x:row r="470">
@@ -7920,16 +7920,16 @@
     </x:row>
     <x:row r="549">
       <x:c r="A549" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B549" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C549" s="1" t="str">
+        <x:v>Perseverance</x:v>
+      </x:c>
+      <x:c r="D549" s="1" t="str">
         <x:v>Усидчивость</x:v>
-      </x:c>
-      <x:c r="D549" s="1" t="str">
-        <x:v>Perseverance</x:v>
       </x:c>
     </x:row>
     <x:row r="550">
@@ -9418,16 +9418,16 @@
     </x:row>
     <x:row r="656">
       <x:c r="A656" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B656" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C656" s="1" t="str">
+        <x:v>Diploma thesis</x:v>
+      </x:c>
+      <x:c r="D656" s="1" t="str">
         <x:v>Дипломная работа</x:v>
-      </x:c>
-      <x:c r="D656" s="1" t="str">
-        <x:v>Diploma thesis</x:v>
       </x:c>
     </x:row>
     <x:row r="657">
@@ -9838,16 +9838,16 @@
     </x:row>
     <x:row r="686">
       <x:c r="A686" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B686" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C686" s="1" t="str">
+        <x:v>confused</x:v>
+      </x:c>
+      <x:c r="D686" s="1" t="str">
         <x:v>растерянно</x:v>
-      </x:c>
-      <x:c r="D686" s="1" t="str">
-        <x:v>confused</x:v>
       </x:c>
     </x:row>
     <x:row r="687">
@@ -12834,16 +12834,16 @@
     </x:row>
     <x:row r="900">
       <x:c r="A900" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B900" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C900" s="1" t="str">
+        <x:v>professional costs</x:v>
+      </x:c>
+      <x:c r="D900" s="1" t="str">
         <x:v>издержки профессии</x:v>
-      </x:c>
-      <x:c r="D900" s="1" t="str">
-        <x:v>professional costs</x:v>
       </x:c>
     </x:row>
     <x:row r="901">
@@ -13044,16 +13044,16 @@
     </x:row>
     <x:row r="915">
       <x:c r="A915" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B915" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C915" s="1" t="str">
+        <x:v>Discharge from the hospital</x:v>
+      </x:c>
+      <x:c r="D915" s="1" t="str">
         <x:v>Выписаться из больницы</x:v>
-      </x:c>
-      <x:c r="D915" s="1" t="str">
-        <x:v>Discharge from the hospital</x:v>
       </x:c>
     </x:row>
     <x:row r="916">
@@ -13926,16 +13926,16 @@
     </x:row>
     <x:row r="978">
       <x:c r="A978" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B978" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C978" s="1" t="str">
+        <x:v>Toothpick</x:v>
+      </x:c>
+      <x:c r="D978" s="1" t="str">
         <x:v>Зубочистка</x:v>
-      </x:c>
-      <x:c r="D978" s="1" t="str">
-        <x:v>Toothpick</x:v>
       </x:c>
     </x:row>
     <x:row r="979">
@@ -14346,30 +14346,30 @@
     </x:row>
     <x:row r="1008">
       <x:c r="A1008" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1008" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1008" s="1" t="str">
+        <x:v>squeamish</x:v>
+      </x:c>
+      <x:c r="D1008" s="1" t="str">
         <x:v>брезгливый</x:v>
-      </x:c>
-      <x:c r="D1008" s="1" t="str">
-        <x:v>squeamish</x:v>
       </x:c>
     </x:row>
     <x:row r="1009">
       <x:c r="A1009" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1009" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1009" s="1" t="str">
+        <x:v>conductor</x:v>
+      </x:c>
+      <x:c r="D1009" s="1" t="str">
         <x:v>проводник</x:v>
-      </x:c>
-      <x:c r="D1009" s="1" t="str">
-        <x:v>conductor</x:v>
       </x:c>
     </x:row>
     <x:row r="1010">
@@ -15704,16 +15704,16 @@
     </x:row>
     <x:row r="1105">
       <x:c r="A1105" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1105" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1105" s="1" t="str">
+        <x:v>Despite</x:v>
+      </x:c>
+      <x:c r="D1105" s="1" t="str">
         <x:v>Не смотря на</x:v>
-      </x:c>
-      <x:c r="D1105" s="1" t="str">
-        <x:v>Despite</x:v>
       </x:c>
     </x:row>
     <x:row r="1106">
@@ -17608,16 +17608,16 @@
     </x:row>
     <x:row r="1241">
       <x:c r="A1241" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1241" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1241" s="1" t="str">
+        <x:v>Activated carbon</x:v>
+      </x:c>
+      <x:c r="D1241" s="1" t="str">
         <x:v>Активированный уголь</x:v>
-      </x:c>
-      <x:c r="D1241" s="1" t="str">
-        <x:v>Activated carbon</x:v>
       </x:c>
     </x:row>
     <x:row r="1242">
@@ -18392,16 +18392,16 @@
     </x:row>
     <x:row r="1297">
       <x:c r="A1297" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1297" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1297" s="1" t="str">
+        <x:v>Pupil</x:v>
+      </x:c>
+      <x:c r="D1297" s="1" t="str">
         <x:v>Зрачек</x:v>
-      </x:c>
-      <x:c r="D1297" s="1" t="str">
-        <x:v>Pupil</x:v>
       </x:c>
     </x:row>
     <x:row r="1298">
@@ -18420,16 +18420,16 @@
     </x:row>
     <x:row r="1299">
       <x:c r="A1299" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1299" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1299" s="1" t="str">
+        <x:v>Picking your nose</x:v>
+      </x:c>
+      <x:c r="D1299" s="1" t="str">
         <x:v>Ковыряться в носу</x:v>
-      </x:c>
-      <x:c r="D1299" s="1" t="str">
-        <x:v>Picking your nose</x:v>
       </x:c>
     </x:row>
     <x:row r="1300">
@@ -20044,16 +20044,16 @@
     </x:row>
     <x:row r="1415">
       <x:c r="A1415" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1415" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1415" s="1" t="str">
+        <x:v>Delay</x:v>
+      </x:c>
+      <x:c r="D1415" s="1" t="str">
         <x:v>Задержка</x:v>
-      </x:c>
-      <x:c r="D1415" s="1" t="str">
-        <x:v>Delay</x:v>
       </x:c>
     </x:row>
     <x:row r="1416">
@@ -20884,16 +20884,16 @@
     </x:row>
     <x:row r="1475">
       <x:c r="A1475" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1475" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1475" s="1" t="str">
+        <x:v>Sage</x:v>
+      </x:c>
+      <x:c r="D1475" s="1" t="str">
         <x:v>Мудрец</x:v>
-      </x:c>
-      <x:c r="D1475" s="1" t="str">
-        <x:v>Sage</x:v>
       </x:c>
     </x:row>
     <x:row r="1476">
@@ -22102,16 +22102,16 @@
     </x:row>
     <x:row r="1562">
       <x:c r="A1562" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1562" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1562" s="1" t="str">
+        <x:v>showcase</x:v>
+      </x:c>
+      <x:c r="D1562" s="1" t="str">
         <x:v>витрина</x:v>
-      </x:c>
-      <x:c r="D1562" s="1" t="str">
-        <x:v>showcase</x:v>
       </x:c>
     </x:row>
     <x:row r="1563">
@@ -23054,16 +23054,16 @@
     </x:row>
     <x:row r="1630">
       <x:c r="A1630" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1630" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1630" s="1" t="str">
+        <x:v>observant</x:v>
+      </x:c>
+      <x:c r="D1630" s="1" t="str">
         <x:v>наблюдательный</x:v>
-      </x:c>
-      <x:c r="D1630" s="1" t="str">
-        <x:v>observant</x:v>
       </x:c>
     </x:row>
     <x:row r="1631">
@@ -23516,16 +23516,16 @@
     </x:row>
     <x:row r="1663">
       <x:c r="A1663" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1663" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1663" s="1" t="str">
+        <x:v>side collection</x:v>
+      </x:c>
+      <x:c r="D1663" s="1" t="str">
         <x:v>побочный сбор</x:v>
-      </x:c>
-      <x:c r="D1663" s="1" t="str">
-        <x:v>side collection</x:v>
       </x:c>
     </x:row>
     <x:row r="1664">
@@ -23642,30 +23642,30 @@
     </x:row>
     <x:row r="1672">
       <x:c r="A1672" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1672" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1672" s="1" t="str">
+        <x:v>Lobe</x:v>
+      </x:c>
+      <x:c r="D1672" s="1" t="str">
         <x:v>Мочка</x:v>
-      </x:c>
-      <x:c r="D1672" s="1" t="str">
-        <x:v>Lobe</x:v>
       </x:c>
     </x:row>
     <x:row r="1673">
       <x:c r="A1673" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1673" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1673" s="1" t="str">
+        <x:v>Earlobe</x:v>
+      </x:c>
+      <x:c r="D1673" s="1" t="str">
         <x:v>Мочка уха</x:v>
-      </x:c>
-      <x:c r="D1673" s="1" t="str">
-        <x:v>Earlobe</x:v>
       </x:c>
     </x:row>
     <x:row r="1674">
@@ -23824,44 +23824,44 @@
     </x:row>
     <x:row r="1685">
       <x:c r="A1685" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1685" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1685" s="1" t="str">
+        <x:v>the decoction has not steeped</x:v>
+      </x:c>
+      <x:c r="D1685" s="1" t="str">
         <x:v>отвар не настоялся</x:v>
-      </x:c>
-      <x:c r="D1685" s="1" t="str">
-        <x:v>the decoction has not steeped</x:v>
       </x:c>
     </x:row>
     <x:row r="1686">
       <x:c r="A1686" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1686" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1686" s="1" t="str">
+        <x:v>Spring</x:v>
+      </x:c>
+      <x:c r="D1686" s="1" t="str">
         <x:v>Пружина</x:v>
-      </x:c>
-      <x:c r="D1686" s="1" t="str">
-        <x:v>Spring</x:v>
       </x:c>
     </x:row>
     <x:row r="1687">
       <x:c r="A1687" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1687" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1687" s="1" t="str">
+        <x:v>Hernia</x:v>
+      </x:c>
+      <x:c r="D1687" s="1" t="str">
         <x:v>Грыжа</x:v>
-      </x:c>
-      <x:c r="D1687" s="1" t="str">
-        <x:v>Hernia</x:v>
       </x:c>
     </x:row>
     <x:row r="1688">
@@ -25196,16 +25196,16 @@
     </x:row>
     <x:row r="1783">
       <x:c r="A1783" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1783" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1783" s="1" t="str">
+        <x:v>Shelter</x:v>
+      </x:c>
+      <x:c r="D1783" s="1" t="str">
         <x:v>Приют</x:v>
-      </x:c>
-      <x:c r="D1783" s="1" t="str">
-        <x:v>Shelter</x:v>
       </x:c>
     </x:row>
     <x:row r="1784">
@@ -26358,16 +26358,16 @@
     </x:row>
     <x:row r="1866">
       <x:c r="A1866" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1866" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1866" s="1" t="str">
+        <x:v>salivation</x:v>
+      </x:c>
+      <x:c r="D1866" s="1" t="str">
         <x:v>слюноотделение</x:v>
-      </x:c>
-      <x:c r="D1866" s="1" t="str">
-        <x:v>salivation</x:v>
       </x:c>
     </x:row>
     <x:row r="1867">
@@ -26428,16 +26428,16 @@
     </x:row>
     <x:row r="1871">
       <x:c r="A1871" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1871" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1871" s="1" t="str">
+        <x:v>injury</x:v>
+      </x:c>
+      <x:c r="D1871" s="1" t="str">
         <x:v>ушиб</x:v>
-      </x:c>
-      <x:c r="D1871" s="1" t="str">
-        <x:v>injury</x:v>
       </x:c>
     </x:row>
     <x:row r="1872">
@@ -27772,16 +27772,16 @@
     </x:row>
     <x:row r="1967">
       <x:c r="A1967" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B1967" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1967" s="1" t="str">
+        <x:v>End justifies the means</x:v>
+      </x:c>
+      <x:c r="D1967" s="1" t="str">
         <x:v>Цель оправдывает средства</x:v>
-      </x:c>
-      <x:c r="D1967" s="1" t="str">
-        <x:v>End justifies the means</x:v>
       </x:c>
     </x:row>
     <x:row r="1968">
@@ -28584,16 +28584,16 @@
     </x:row>
     <x:row r="2025">
       <x:c r="A2025" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2025" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2025" s="1" t="str">
+        <x:v>Toad</x:v>
+      </x:c>
+      <x:c r="D2025" s="1" t="str">
         <x:v>Жаба</x:v>
-      </x:c>
-      <x:c r="D2025" s="1" t="str">
-        <x:v>Toad</x:v>
       </x:c>
     </x:row>
     <x:row r="2026">
@@ -28612,16 +28612,16 @@
     </x:row>
     <x:row r="2027">
       <x:c r="A2027" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2027" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2027" s="1" t="str">
+        <x:v>Don't bother me with this.</x:v>
+      </x:c>
+      <x:c r="D2027" s="1" t="str">
         <x:v>Не доставай меня с этим</x:v>
-      </x:c>
-      <x:c r="D2027" s="1" t="str">
-        <x:v>Don't bother me with this.</x:v>
       </x:c>
     </x:row>
     <x:row r="2028">
@@ -28934,16 +28934,16 @@
     </x:row>
     <x:row r="2050">
       <x:c r="A2050" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2050" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2050" s="1" t="str">
+        <x:v>cardboard</x:v>
+      </x:c>
+      <x:c r="D2050" s="1" t="str">
         <x:v>картон</x:v>
-      </x:c>
-      <x:c r="D2050" s="1" t="str">
-        <x:v>cardboard</x:v>
       </x:c>
     </x:row>
     <x:row r="2051">
@@ -28990,16 +28990,16 @@
     </x:row>
     <x:row r="2054">
       <x:c r="A2054" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2054" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2054" s="1" t="str">
+        <x:v>I give up</x:v>
+      </x:c>
+      <x:c r="D2054" s="1" t="str">
         <x:v>я сдаюсь</x:v>
-      </x:c>
-      <x:c r="D2054" s="1" t="str">
-        <x:v>I give up</x:v>
       </x:c>
     </x:row>
     <x:row r="2055">
@@ -30530,16 +30530,16 @@
     </x:row>
     <x:row r="2164">
       <x:c r="A2164" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2164" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2164" s="1" t="str">
+        <x:v>unlike people</x:v>
+      </x:c>
+      <x:c r="D2164" s="1" t="str">
         <x:v>в отличие от людей</x:v>
-      </x:c>
-      <x:c r="D2164" s="1" t="str">
-        <x:v>unlike people</x:v>
       </x:c>
     </x:row>
     <x:row r="2165">
@@ -30950,16 +30950,16 @@
     </x:row>
     <x:row r="2194">
       <x:c r="A2194" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2194" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2194" s="1" t="str">
+        <x:v>Mountain Range</x:v>
+      </x:c>
+      <x:c r="D2194" s="1" t="str">
         <x:v>Горный Хребет</x:v>
-      </x:c>
-      <x:c r="D2194" s="1" t="str">
-        <x:v>Mountain Range</x:v>
       </x:c>
     </x:row>
     <x:row r="2195">
@@ -32770,16 +32770,16 @@
     </x:row>
     <x:row r="2324">
       <x:c r="A2324" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2324" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2324" s="1" t="str">
+        <x:v>Comparison</x:v>
+      </x:c>
+      <x:c r="D2324" s="1" t="str">
         <x:v>Сравнение</x:v>
-      </x:c>
-      <x:c r="D2324" s="1" t="str">
-        <x:v>Comparison</x:v>
       </x:c>
     </x:row>
     <x:row r="2325">
@@ -33372,16 +33372,16 @@
     </x:row>
     <x:row r="2367">
       <x:c r="A2367" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2367" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2367" s="1" t="str">
+        <x:v>automation</x:v>
+      </x:c>
+      <x:c r="D2367" s="1" t="str">
         <x:v>автоматизация</x:v>
-      </x:c>
-      <x:c r="D2367" s="1" t="str">
-        <x:v>automation</x:v>
       </x:c>
     </x:row>
     <x:row r="2368">
@@ -33442,16 +33442,16 @@
     </x:row>
     <x:row r="2372">
       <x:c r="A2372" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2372" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2372" s="1" t="str">
+        <x:v>Coffee lid</x:v>
+      </x:c>
+      <x:c r="D2372" s="1" t="str">
         <x:v>Крышка для кофе</x:v>
-      </x:c>
-      <x:c r="D2372" s="1" t="str">
-        <x:v>Coffee lid</x:v>
       </x:c>
     </x:row>
     <x:row r="2373">
@@ -33540,16 +33540,16 @@
     </x:row>
     <x:row r="2379">
       <x:c r="A2379" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2379" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2379" s="1" t="str">
+        <x:v>Boar</x:v>
+      </x:c>
+      <x:c r="D2379" s="1" t="str">
         <x:v>Кабан</x:v>
-      </x:c>
-      <x:c r="D2379" s="1" t="str">
-        <x:v>Boar</x:v>
       </x:c>
     </x:row>
     <x:row r="2380">
@@ -34450,16 +34450,16 @@
     </x:row>
     <x:row r="2444">
       <x:c r="A2444" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2444" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2444" s="1" t="str">
+        <x:v>avoid</x:v>
+      </x:c>
+      <x:c r="D2444" s="1" t="str">
         <x:v>избегать</x:v>
-      </x:c>
-      <x:c r="D2444" s="1" t="str">
-        <x:v>avoid</x:v>
       </x:c>
     </x:row>
     <x:row r="2445">
@@ -34646,16 +34646,16 @@
     </x:row>
     <x:row r="2458">
       <x:c r="A2458" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2458" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2458" s="1" t="str">
+        <x:v>booger in the nose</x:v>
+      </x:c>
+      <x:c r="D2458" s="1" t="str">
         <x:v>козявка в носу</x:v>
-      </x:c>
-      <x:c r="D2458" s="1" t="str">
-        <x:v>booger in the nose</x:v>
       </x:c>
     </x:row>
     <x:row r="2459">
@@ -34856,16 +34856,16 @@
     </x:row>
     <x:row r="2473">
       <x:c r="A2473" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2473" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2473" s="1" t="str">
+        <x:v>it seemed to me</x:v>
+      </x:c>
+      <x:c r="D2473" s="1" t="str">
         <x:v>показалось мне</x:v>
-      </x:c>
-      <x:c r="D2473" s="1" t="str">
-        <x:v>it seemed to me</x:v>
       </x:c>
     </x:row>
     <x:row r="2474">
@@ -35080,16 +35080,16 @@
     </x:row>
     <x:row r="2489">
       <x:c r="A2489" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2489" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2489" s="1" t="str">
+        <x:v>Boast</x:v>
+      </x:c>
+      <x:c r="D2489" s="1" t="str">
         <x:v>Хвастаться</x:v>
-      </x:c>
-      <x:c r="D2489" s="1" t="str">
-        <x:v>Boast</x:v>
       </x:c>
     </x:row>
     <x:row r="2490">
@@ -35122,16 +35122,16 @@
     </x:row>
     <x:row r="2492">
       <x:c r="A2492" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2492" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2492" s="1" t="str">
+        <x:v>Breed</x:v>
+      </x:c>
+      <x:c r="D2492" s="1" t="str">
         <x:v>Порода</x:v>
-      </x:c>
-      <x:c r="D2492" s="1" t="str">
-        <x:v>Breed</x:v>
       </x:c>
     </x:row>
     <x:row r="2493">
@@ -35920,16 +35920,16 @@
     </x:row>
     <x:row r="2549">
       <x:c r="A2549" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2549" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2549" s="1" t="str">
+        <x:v>Angle</x:v>
+      </x:c>
+      <x:c r="D2549" s="1" t="str">
         <x:v>Ракурс</x:v>
-      </x:c>
-      <x:c r="D2549" s="1" t="str">
-        <x:v>Angle</x:v>
       </x:c>
     </x:row>
     <x:row r="2550">
@@ -37040,16 +37040,16 @@
     </x:row>
     <x:row r="2629">
       <x:c r="A2629" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2629" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2629" s="1" t="str">
+        <x:v>It's gone too far</x:v>
+      </x:c>
+      <x:c r="D2629" s="1" t="str">
         <x:v>Это зашло слишком далеко</x:v>
-      </x:c>
-      <x:c r="D2629" s="1" t="str">
-        <x:v>It's gone too far</x:v>
       </x:c>
     </x:row>
     <x:row r="2630">
@@ -37180,16 +37180,16 @@
     </x:row>
     <x:row r="2639">
       <x:c r="A2639" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2639" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2639" s="1" t="str">
+        <x:v>It just seems this way to you</x:v>
+      </x:c>
+      <x:c r="D2639" s="1" t="str">
         <x:v>Тебе кажется</x:v>
-      </x:c>
-      <x:c r="D2639" s="1" t="str">
-        <x:v>It just seems this way to you</x:v>
       </x:c>
     </x:row>
     <x:row r="2640">
@@ -37208,16 +37208,16 @@
     </x:row>
     <x:row r="2641">
       <x:c r="A2641" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2641" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2641" s="1" t="str">
+        <x:v>Carbohydrates</x:v>
+      </x:c>
+      <x:c r="D2641" s="1" t="str">
         <x:v>Углеводы</x:v>
-      </x:c>
-      <x:c r="D2641" s="1" t="str">
-        <x:v>Carbohydrates</x:v>
       </x:c>
     </x:row>
     <x:row r="2642">
@@ -37306,16 +37306,16 @@
     </x:row>
     <x:row r="2648">
       <x:c r="A2648" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2648" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2648" s="1" t="str">
+        <x:v>Jay</x:v>
+      </x:c>
+      <x:c r="D2648" s="1" t="str">
         <x:v>Сойка</x:v>
-      </x:c>
-      <x:c r="D2648" s="1" t="str">
-        <x:v>Jay</x:v>
       </x:c>
     </x:row>
     <x:row r="2649">
@@ -37418,16 +37418,16 @@
     </x:row>
     <x:row r="2656">
       <x:c r="A2656" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2656" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2656" s="1" t="str">
+        <x:v>Envelope</x:v>
+      </x:c>
+      <x:c r="D2656" s="1" t="str">
         <x:v>Конверт</x:v>
-      </x:c>
-      <x:c r="D2656" s="1" t="str">
-        <x:v>Envelope</x:v>
       </x:c>
     </x:row>
     <x:row r="2657">
@@ -37656,16 +37656,16 @@
     </x:row>
     <x:row r="2673">
       <x:c r="A2673" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2673" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2673" s="1" t="str">
+        <x:v>close the curtains</x:v>
+      </x:c>
+      <x:c r="D2673" s="1" t="str">
         <x:v>зашторить шторы</x:v>
-      </x:c>
-      <x:c r="D2673" s="1" t="str">
-        <x:v>close the curtains</x:v>
       </x:c>
     </x:row>
     <x:row r="2674">
@@ -37880,16 +37880,16 @@
     </x:row>
     <x:row r="2689">
       <x:c r="A2689" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2689" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2689" s="1" t="str">
+        <x:v>Tarot spread</x:v>
+      </x:c>
+      <x:c r="D2689" s="1" t="str">
         <x:v>Расклад таро</x:v>
-      </x:c>
-      <x:c r="D2689" s="1" t="str">
-        <x:v>Tarot spread</x:v>
       </x:c>
     </x:row>
     <x:row r="2690">
@@ -38202,16 +38202,16 @@
     </x:row>
     <x:row r="2712">
       <x:c r="A2712" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2712" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2712" s="1" t="str">
+        <x:v>Mineral fertilizer</x:v>
+      </x:c>
+      <x:c r="D2712" s="1" t="str">
         <x:v>Минеральное удобрение</x:v>
-      </x:c>
-      <x:c r="D2712" s="1" t="str">
-        <x:v>Mineral fertilizer</x:v>
       </x:c>
     </x:row>
     <x:row r="2713">
@@ -38384,16 +38384,16 @@
     </x:row>
     <x:row r="2725">
       <x:c r="A2725" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2725" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2725" s="1" t="str">
+        <x:v>Beekeeping</x:v>
+      </x:c>
+      <x:c r="D2725" s="1" t="str">
         <x:v>Пчеловодство</x:v>
-      </x:c>
-      <x:c r="D2725" s="1" t="str">
-        <x:v>Beekeeping</x:v>
       </x:c>
     </x:row>
     <x:row r="2726">
@@ -38426,16 +38426,16 @@
     </x:row>
     <x:row r="2728">
       <x:c r="A2728" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2728" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2728" s="1" t="str">
+        <x:v>puddle</x:v>
+      </x:c>
+      <x:c r="D2728" s="1" t="str">
         <x:v>лужа</x:v>
-      </x:c>
-      <x:c r="D2728" s="1" t="str">
-        <x:v>puddle</x:v>
       </x:c>
     </x:row>
     <x:row r="2729">
@@ -38468,16 +38468,16 @@
     </x:row>
     <x:row r="2731">
       <x:c r="A2731" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B2731" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2731" s="1" t="str">
+        <x:v>ჩემი გაჩერება</x:v>
+      </x:c>
+      <x:c r="D2731" s="1" t="str">
         <x:v>моя остановка</x:v>
-      </x:c>
-      <x:c r="D2731" s="1" t="str">
-        <x:v>ჩემი გაჩერება</x:v>
       </x:c>
     </x:row>
     <x:row r="2732">
@@ -38664,16 +38664,16 @@
     </x:row>
     <x:row r="2745">
       <x:c r="A2745" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2745" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2745" s="1" t="str">
+        <x:v>preventive examination</x:v>
+      </x:c>
+      <x:c r="D2745" s="1" t="str">
         <x:v>профилактический осмотр</x:v>
-      </x:c>
-      <x:c r="D2745" s="1" t="str">
-        <x:v>preventive examination</x:v>
       </x:c>
     </x:row>
     <x:row r="2746">
@@ -38958,16 +38958,16 @@
     </x:row>
     <x:row r="2766">
       <x:c r="A2766" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2766" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2766" s="1" t="str">
+        <x:v>do you want to argue?</x:v>
+      </x:c>
+      <x:c r="D2766" s="1" t="str">
         <x:v>ты хочешь поспорить?</x:v>
-      </x:c>
-      <x:c r="D2766" s="1" t="str">
-        <x:v>do you want to argue?</x:v>
       </x:c>
     </x:row>
     <x:row r="2767">
@@ -38986,16 +38986,16 @@
     </x:row>
     <x:row r="2768">
       <x:c r="A2768" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2768" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2768" s="1" t="str">
+        <x:v>how long is the commercial before the movie?</x:v>
+      </x:c>
+      <x:c r="D2768" s="1" t="str">
         <x:v>сколько длится реклама перед фильмом</x:v>
-      </x:c>
-      <x:c r="D2768" s="1" t="str">
-        <x:v>how long is the commercial before the movie?</x:v>
       </x:c>
     </x:row>
     <x:row r="2769">
@@ -39476,16 +39476,16 @@
     </x:row>
     <x:row r="2803">
       <x:c r="A2803" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2803" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2803" s="1" t="str">
+        <x:v>I can't stand it</x:v>
+      </x:c>
+      <x:c r="D2803" s="1" t="str">
         <x:v>Я этого не выношу</x:v>
-      </x:c>
-      <x:c r="D2803" s="1" t="str">
-        <x:v>I can't stand it</x:v>
       </x:c>
     </x:row>
     <x:row r="2804">
@@ -39532,16 +39532,16 @@
     </x:row>
     <x:row r="2807">
       <x:c r="A2807" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2807" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2807" s="1" t="str">
+        <x:v>tense</x:v>
+      </x:c>
+      <x:c r="D2807" s="1" t="str">
         <x:v>напряжен</x:v>
-      </x:c>
-      <x:c r="D2807" s="1" t="str">
-        <x:v>tense</x:v>
       </x:c>
     </x:row>
     <x:row r="2808">
@@ -39714,16 +39714,16 @@
     </x:row>
     <x:row r="2820">
       <x:c r="A2820" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2820" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2820" s="1" t="str">
+        <x:v>meander</x:v>
+      </x:c>
+      <x:c r="D2820" s="1" t="str">
         <x:v>петлять</x:v>
-      </x:c>
-      <x:c r="D2820" s="1" t="str">
-        <x:v>meander</x:v>
       </x:c>
     </x:row>
     <x:row r="2821">
@@ -40134,16 +40134,16 @@
     </x:row>
     <x:row r="2850">
       <x:c r="A2850" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2850" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2850" s="1" t="str">
+        <x:v>I have omitted unnecessary details in the description</x:v>
+      </x:c>
+      <x:c r="D2850" s="1" t="str">
         <x:v>Я опустил ненужные подробности в описании</x:v>
-      </x:c>
-      <x:c r="D2850" s="1" t="str">
-        <x:v>I have omitted unnecessary details in the description</x:v>
       </x:c>
     </x:row>
     <x:row r="2851">
@@ -40316,16 +40316,16 @@
     </x:row>
     <x:row r="2863">
       <x:c r="A2863" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2863" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2863" s="1" t="str">
+        <x:v>What do they advise?</x:v>
+      </x:c>
+      <x:c r="D2863" s="1" t="str">
         <x:v>Что советуют</x:v>
-      </x:c>
-      <x:c r="D2863" s="1" t="str">
-        <x:v>What do they advise?</x:v>
       </x:c>
     </x:row>
     <x:row r="2864">
@@ -41002,16 +41002,16 @@
     </x:row>
     <x:row r="2912">
       <x:c r="A2912" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2912" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2912" s="1" t="str">
+        <x:v>maggot</x:v>
+      </x:c>
+      <x:c r="D2912" s="1" t="str">
         <x:v>опарыш</x:v>
-      </x:c>
-      <x:c r="D2912" s="1" t="str">
-        <x:v>maggot</x:v>
       </x:c>
     </x:row>
     <x:row r="2913">
@@ -41926,16 +41926,16 @@
     </x:row>
     <x:row r="2978">
       <x:c r="A2978" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2978" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2978" s="1" t="str">
+        <x:v>Literary translation</x:v>
+      </x:c>
+      <x:c r="D2978" s="1" t="str">
         <x:v>Художественный перевод</x:v>
-      </x:c>
-      <x:c r="D2978" s="1" t="str">
-        <x:v>Literary translation</x:v>
       </x:c>
     </x:row>
     <x:row r="2979">
@@ -42206,16 +42206,16 @@
     </x:row>
     <x:row r="2998">
       <x:c r="A2998" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B2998" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2998" s="1" t="str">
+        <x:v>buttocks</x:v>
+      </x:c>
+      <x:c r="D2998" s="1" t="str">
         <x:v>ягодицы</x:v>
-      </x:c>
-      <x:c r="D2998" s="1" t="str">
-        <x:v>buttocks</x:v>
       </x:c>
     </x:row>
     <x:row r="2999">
@@ -42304,16 +42304,16 @@
     </x:row>
     <x:row r="3005">
       <x:c r="A3005" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3005" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3005" s="1" t="str">
+        <x:v>cutlery</x:v>
+      </x:c>
+      <x:c r="D3005" s="1" t="str">
         <x:v>соловые приборы</x:v>
-      </x:c>
-      <x:c r="D3005" s="1" t="str">
-        <x:v>cutlery</x:v>
       </x:c>
     </x:row>
     <x:row r="3006">
@@ -42710,16 +42710,16 @@
     </x:row>
     <x:row r="3034">
       <x:c r="A3034" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3034" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3034" s="1" t="str">
+        <x:v>Cardboard</x:v>
+      </x:c>
+      <x:c r="D3034" s="1" t="str">
         <x:v>Картон</x:v>
-      </x:c>
-      <x:c r="D3034" s="1" t="str">
-        <x:v>Cardboard</x:v>
       </x:c>
     </x:row>
     <x:row r="3035">
@@ -43942,16 +43942,16 @@
     </x:row>
     <x:row r="3122">
       <x:c r="A3122" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3122" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3122" s="1" t="str">
+        <x:v>awkward</x:v>
+      </x:c>
+      <x:c r="D3122" s="1" t="str">
         <x:v>Неловко</x:v>
-      </x:c>
-      <x:c r="D3122" s="1" t="str">
-        <x:v>awkward</x:v>
       </x:c>
     </x:row>
     <x:row r="3123">
@@ -44250,16 +44250,16 @@
     </x:row>
     <x:row r="3144">
       <x:c r="A3144" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3144" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3144" s="1" t="str">
+        <x:v>Cost price</x:v>
+      </x:c>
+      <x:c r="D3144" s="1" t="str">
         <x:v>Себестоимость</x:v>
-      </x:c>
-      <x:c r="D3144" s="1" t="str">
-        <x:v>Cost price</x:v>
       </x:c>
     </x:row>
     <x:row r="3145">
@@ -44278,16 +44278,16 @@
     </x:row>
     <x:row r="3146">
       <x:c r="A3146" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3146" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3146" s="1" t="str">
+        <x:v>Gas stove</x:v>
+      </x:c>
+      <x:c r="D3146" s="1" t="str">
         <x:v>Газовая плита</x:v>
-      </x:c>
-      <x:c r="D3146" s="1" t="str">
-        <x:v>Gas stove</x:v>
       </x:c>
     </x:row>
     <x:row r="3147">
@@ -45048,16 +45048,16 @@
     </x:row>
     <x:row r="3201">
       <x:c r="A3201" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3201" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3201" s="1" t="str">
+        <x:v>Active substance</x:v>
+      </x:c>
+      <x:c r="D3201" s="1" t="str">
         <x:v>Действующее вещество</x:v>
-      </x:c>
-      <x:c r="D3201" s="1" t="str">
-        <x:v>Active substance</x:v>
       </x:c>
     </x:row>
     <x:row r="3202">
@@ -45090,30 +45090,30 @@
     </x:row>
     <x:row r="3204">
       <x:c r="A3204" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3204" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3204" s="1" t="str">
+        <x:v>ჯანჯაფილი</x:v>
+      </x:c>
+      <x:c r="D3204" s="1" t="str">
         <x:v>Имбирь</x:v>
-      </x:c>
-      <x:c r="D3204" s="1" t="str">
-        <x:v>ჯანჯაფილი</x:v>
       </x:c>
     </x:row>
     <x:row r="3205">
       <x:c r="A3205" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3205" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3205" s="1" t="str">
+        <x:v>Offense</x:v>
+      </x:c>
+      <x:c r="D3205" s="1" t="str">
         <x:v>Правонарушение</x:v>
-      </x:c>
-      <x:c r="D3205" s="1" t="str">
-        <x:v>Offense</x:v>
       </x:c>
     </x:row>
     <x:row r="3206">
@@ -45146,30 +45146,30 @@
     </x:row>
     <x:row r="3208">
       <x:c r="A3208" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3208" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3208" s="1" t="str">
+        <x:v>არ არის ელექტროენერგია</x:v>
+      </x:c>
+      <x:c r="D3208" s="1" t="str">
         <x:v>электричества нет</x:v>
-      </x:c>
-      <x:c r="D3208" s="1" t="str">
-        <x:v>არ არის ელექტროენერგია</x:v>
       </x:c>
     </x:row>
     <x:row r="3209">
       <x:c r="A3209" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3209" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3209" s="1" t="str">
+        <x:v>შენც არ გაქვს დენი?</x:v>
+      </x:c>
+      <x:c r="D3209" s="1" t="str">
         <x:v>у вас тоже нет электричества?</x:v>
-      </x:c>
-      <x:c r="D3209" s="1" t="str">
-        <x:v>შენც არ გაქვს დენი?</x:v>
       </x:c>
     </x:row>
     <x:row r="3210">
@@ -45468,16 +45468,16 @@
     </x:row>
     <x:row r="3231">
       <x:c r="A3231" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3231" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3231" s="1" t="str">
+        <x:v>Wasp</x:v>
+      </x:c>
+      <x:c r="D3231" s="1" t="str">
         <x:v>Оса</x:v>
-      </x:c>
-      <x:c r="D3231" s="1" t="str">
-        <x:v>Wasp</x:v>
       </x:c>
     </x:row>
     <x:row r="3232">
@@ -45524,16 +45524,16 @@
     </x:row>
     <x:row r="3235">
       <x:c r="A3235" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3235" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3235" s="1" t="str">
+        <x:v>Help yourself</x:v>
+      </x:c>
+      <x:c r="D3235" s="1" t="str">
         <x:v>Угощайтесь</x:v>
-      </x:c>
-      <x:c r="D3235" s="1" t="str">
-        <x:v>Help yourself</x:v>
       </x:c>
     </x:row>
     <x:row r="3236">
@@ -45552,16 +45552,16 @@
     </x:row>
     <x:row r="3237">
       <x:c r="A3237" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3237" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3237" s="1" t="str">
+        <x:v>Mantle</x:v>
+      </x:c>
+      <x:c r="D3237" s="1" t="str">
         <x:v>Мантия</x:v>
-      </x:c>
-      <x:c r="D3237" s="1" t="str">
-        <x:v>Mantle</x:v>
       </x:c>
     </x:row>
     <x:row r="3238">
@@ -45594,16 +45594,16 @@
     </x:row>
     <x:row r="3240">
       <x:c r="A3240" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3240" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3240" s="1" t="str">
+        <x:v>combing</x:v>
+      </x:c>
+      <x:c r="D3240" s="1" t="str">
         <x:v>Рассчесывать</x:v>
-      </x:c>
-      <x:c r="D3240" s="1" t="str">
-        <x:v>combing</x:v>
       </x:c>
     </x:row>
     <x:row r="3241">
@@ -45636,16 +45636,16 @@
     </x:row>
     <x:row r="3243">
       <x:c r="A3243" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3243" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3243" s="1" t="str">
+        <x:v>Pleased</x:v>
+      </x:c>
+      <x:c r="D3243" s="1" t="str">
         <x:v>Довольный</x:v>
-      </x:c>
-      <x:c r="D3243" s="1" t="str">
-        <x:v>Pleased</x:v>
       </x:c>
     </x:row>
     <x:row r="3244">
@@ -45874,44 +45874,44 @@
     </x:row>
     <x:row r="3260">
       <x:c r="A3260" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3260" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3260" s="1" t="str">
+        <x:v>Socket</x:v>
+      </x:c>
+      <x:c r="D3260" s="1" t="str">
         <x:v>Розетка</x:v>
-      </x:c>
-      <x:c r="D3260" s="1" t="str">
-        <x:v>Socket</x:v>
       </x:c>
     </x:row>
     <x:row r="3261">
       <x:c r="A3261" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3261" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3261" s="1" t="str">
+        <x:v>Loose</x:v>
+      </x:c>
+      <x:c r="D3261" s="1" t="str">
         <x:v>Рыхлый</x:v>
-      </x:c>
-      <x:c r="D3261" s="1" t="str">
-        <x:v>Loose</x:v>
       </x:c>
     </x:row>
     <x:row r="3262">
       <x:c r="A3262" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3262" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3262" s="1" t="str">
+        <x:v>flabby</x:v>
+      </x:c>
+      <x:c r="D3262" s="1" t="str">
         <x:v>Дрябоый</x:v>
-      </x:c>
-      <x:c r="D3262" s="1" t="str">
-        <x:v>flabby</x:v>
       </x:c>
     </x:row>
     <x:row r="3263">
@@ -45958,16 +45958,16 @@
     </x:row>
     <x:row r="3266">
       <x:c r="A3266" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3266" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3266" s="1" t="str">
+        <x:v>What is it made of?</x:v>
+      </x:c>
+      <x:c r="D3266" s="1" t="str">
         <x:v>Из чего это сделано?</x:v>
-      </x:c>
-      <x:c r="D3266" s="1" t="str">
-        <x:v>What is it made of?</x:v>
       </x:c>
     </x:row>
     <x:row r="3267">
@@ -46126,16 +46126,16 @@
     </x:row>
     <x:row r="3278">
       <x:c r="A3278" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3278" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3278" s="1" t="str">
+        <x:v>hike</x:v>
+      </x:c>
+      <x:c r="D3278" s="1" t="str">
         <x:v>Поход</x:v>
-      </x:c>
-      <x:c r="D3278" s="1" t="str">
-        <x:v>hike</x:v>
       </x:c>
     </x:row>
     <x:row r="3279">
@@ -46280,30 +46280,30 @@
     </x:row>
     <x:row r="3289">
       <x:c r="A3289" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3289" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3289" s="1" t="str">
+        <x:v>Pass tests</x:v>
+      </x:c>
+      <x:c r="D3289" s="1" t="str">
         <x:v>Сдать анализы</x:v>
-      </x:c>
-      <x:c r="D3289" s="1" t="str">
-        <x:v>Pass tests</x:v>
       </x:c>
     </x:row>
     <x:row r="3290">
       <x:c r="A3290" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3290" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3290" s="1" t="str">
+        <x:v>Hairstyle</x:v>
+      </x:c>
+      <x:c r="D3290" s="1" t="str">
         <x:v>Причёска</x:v>
-      </x:c>
-      <x:c r="D3290" s="1" t="str">
-        <x:v>Hairstyle</x:v>
       </x:c>
     </x:row>
     <x:row r="3291">
@@ -47064,44 +47064,44 @@
     </x:row>
     <x:row r="3345">
       <x:c r="A3345" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3345" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3345" s="1" t="str">
+        <x:v>humus</x:v>
+      </x:c>
+      <x:c r="D3345" s="1" t="str">
         <x:v>перегной</x:v>
-      </x:c>
-      <x:c r="D3345" s="1" t="str">
-        <x:v>humus</x:v>
       </x:c>
     </x:row>
     <x:row r="3346">
       <x:c r="A3346" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3346" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3346" s="1" t="str">
+        <x:v>Manure</x:v>
+      </x:c>
+      <x:c r="D3346" s="1" t="str">
         <x:v>Навоз</x:v>
-      </x:c>
-      <x:c r="D3346" s="1" t="str">
-        <x:v>Manure</x:v>
       </x:c>
     </x:row>
     <x:row r="3347">
       <x:c r="A3347" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3347" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3347" s="1" t="str">
+        <x:v>ამანათის ნომერი ორმოცდაათი</x:v>
+      </x:c>
+      <x:c r="D3347" s="1" t="str">
         <x:v>посылка номер пятьдесят</x:v>
-      </x:c>
-      <x:c r="D3347" s="1" t="str">
-        <x:v>ამანათის ნომერი ორმოცდაათი</x:v>
       </x:c>
     </x:row>
     <x:row r="3348">
@@ -47218,16 +47218,16 @@
     </x:row>
     <x:row r="3356">
       <x:c r="A3356" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3356" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3356" s="1" t="str">
+        <x:v>ექვსი</x:v>
+      </x:c>
+      <x:c r="D3356" s="1" t="str">
         <x:v>шесть</x:v>
-      </x:c>
-      <x:c r="D3356" s="1" t="str">
-        <x:v>ექვსი</x:v>
       </x:c>
     </x:row>
     <x:row r="3357">
@@ -47260,16 +47260,16 @@
     </x:row>
     <x:row r="3359">
       <x:c r="A3359" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3359" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3359" s="1" t="str">
+        <x:v>ground</x:v>
+      </x:c>
+      <x:c r="D3359" s="1" t="str">
         <x:v>молотый</x:v>
-      </x:c>
-      <x:c r="D3359" s="1" t="str">
-        <x:v>ground</x:v>
       </x:c>
     </x:row>
     <x:row r="3360">
@@ -47456,16 +47456,16 @@
     </x:row>
     <x:row r="3373">
       <x:c r="A3373" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3373" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3373" s="1" t="str">
+        <x:v>აქ დავჯდები</x:v>
+      </x:c>
+      <x:c r="D3373" s="1" t="str">
         <x:v>я сяду тут</x:v>
-      </x:c>
-      <x:c r="D3373" s="1" t="str">
-        <x:v>აქ დავჯდები</x:v>
       </x:c>
     </x:row>
     <x:row r="3374">
@@ -47862,72 +47862,72 @@
     </x:row>
     <x:row r="3402">
       <x:c r="A3402" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3402" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3402" s="1" t="str">
+        <x:v>flattery</x:v>
+      </x:c>
+      <x:c r="D3402" s="1" t="str">
         <x:v>лесть</x:v>
-      </x:c>
-      <x:c r="D3402" s="1" t="str">
-        <x:v>flattery</x:v>
       </x:c>
     </x:row>
     <x:row r="3403">
       <x:c r="A3403" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3403" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3403" s="1" t="str">
+        <x:v>terrace</x:v>
+      </x:c>
+      <x:c r="D3403" s="1" t="str">
         <x:v>терасса</x:v>
-      </x:c>
-      <x:c r="D3403" s="1" t="str">
-        <x:v>terrace</x:v>
       </x:c>
     </x:row>
     <x:row r="3404">
       <x:c r="A3404" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3404" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3404" s="1" t="str">
+        <x:v>Hut</x:v>
+      </x:c>
+      <x:c r="D3404" s="1" t="str">
         <x:v>Хижина</x:v>
-      </x:c>
-      <x:c r="D3404" s="1" t="str">
-        <x:v>Hut</x:v>
       </x:c>
     </x:row>
     <x:row r="3405">
       <x:c r="A3405" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3405" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3405" s="1" t="str">
+        <x:v>ceiling</x:v>
+      </x:c>
+      <x:c r="D3405" s="1" t="str">
         <x:v>потолок</x:v>
-      </x:c>
-      <x:c r="D3405" s="1" t="str">
-        <x:v>ceiling</x:v>
       </x:c>
     </x:row>
     <x:row r="3406">
       <x:c r="A3406" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3406" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3406" s="1" t="str">
+        <x:v>attic</x:v>
+      </x:c>
+      <x:c r="D3406" s="1" t="str">
         <x:v>чердак</x:v>
-      </x:c>
-      <x:c r="D3406" s="1" t="str">
-        <x:v>attic</x:v>
       </x:c>
     </x:row>
     <x:row r="3407">
@@ -48170,16 +48170,16 @@
     </x:row>
     <x:row r="3424">
       <x:c r="A3424" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3424" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3424" s="1" t="str">
+        <x:v>სად არის ნაგავი?</x:v>
+      </x:c>
+      <x:c r="D3424" s="1" t="str">
         <x:v>в где мусорка?</x:v>
-      </x:c>
-      <x:c r="D3424" s="1" t="str">
-        <x:v>სად არის ნაგავი?</x:v>
       </x:c>
     </x:row>
     <x:row r="3425">
@@ -49122,16 +49122,16 @@
     </x:row>
     <x:row r="3492">
       <x:c r="A3492" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3492" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3492" s="1" t="str">
+        <x:v>seal</x:v>
+      </x:c>
+      <x:c r="D3492" s="1" t="str">
         <x:v>тюлень</x:v>
-      </x:c>
-      <x:c r="D3492" s="1" t="str">
-        <x:v>seal</x:v>
       </x:c>
     </x:row>
     <x:row r="3493">
@@ -49248,72 +49248,72 @@
     </x:row>
     <x:row r="3501">
       <x:c r="A3501" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3501" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3501" s="1" t="str">
+        <x:v>ხუთი</x:v>
+      </x:c>
+      <x:c r="D3501" s="1" t="str">
         <x:v>пять</x:v>
-      </x:c>
-      <x:c r="D3501" s="1" t="str">
-        <x:v>ხუთი</x:v>
       </x:c>
     </x:row>
     <x:row r="3502">
       <x:c r="A3502" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3502" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3502" s="1" t="str">
+        <x:v>ცხრა</x:v>
+      </x:c>
+      <x:c r="D3502" s="1" t="str">
         <x:v>девять</x:v>
-      </x:c>
-      <x:c r="D3502" s="1" t="str">
-        <x:v>ცხრა</x:v>
       </x:c>
     </x:row>
     <x:row r="3503">
       <x:c r="A3503" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3503" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3503" s="1" t="str">
+        <x:v>ჩვენება</x:v>
+      </x:c>
+      <x:c r="D3503" s="1" t="str">
         <x:v>покажите</x:v>
-      </x:c>
-      <x:c r="D3503" s="1" t="str">
-        <x:v>ჩვენება</x:v>
       </x:c>
     </x:row>
     <x:row r="3504">
       <x:c r="A3504" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3504" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3504" s="1" t="str">
+        <x:v>სასაჩუქრე ჩანთა</x:v>
+      </x:c>
+      <x:c r="D3504" s="1" t="str">
         <x:v>подарочный пакет</x:v>
-      </x:c>
-      <x:c r="D3504" s="1" t="str">
-        <x:v>სასაჩუქრე ჩანთა</x:v>
       </x:c>
     </x:row>
     <x:row r="3505">
       <x:c r="A3505" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3505" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3505" s="1" t="str">
+        <x:v>consistent</x:v>
+      </x:c>
+      <x:c r="D3505" s="1" t="str">
         <x:v>последовательный</x:v>
-      </x:c>
-      <x:c r="D3505" s="1" t="str">
-        <x:v>consistent</x:v>
       </x:c>
     </x:row>
     <x:row r="3506">
@@ -49360,16 +49360,16 @@
     </x:row>
     <x:row r="3509">
       <x:c r="A3509" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3509" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3509" s="1" t="str">
+        <x:v>ქათამი</x:v>
+      </x:c>
+      <x:c r="D3509" s="1" t="str">
         <x:v>куриный</x:v>
-      </x:c>
-      <x:c r="D3509" s="1" t="str">
-        <x:v>ქათამი</x:v>
       </x:c>
     </x:row>
     <x:row r="3510">
@@ -49444,16 +49444,16 @@
     </x:row>
     <x:row r="3515">
       <x:c r="A3515" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3515" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3515" s="1" t="str">
+        <x:v>საფერფლე</x:v>
+      </x:c>
+      <x:c r="D3515" s="1" t="str">
         <x:v>пепельница</x:v>
-      </x:c>
-      <x:c r="D3515" s="1" t="str">
-        <x:v>საფერფლე</x:v>
       </x:c>
     </x:row>
     <x:row r="3516">
@@ -49472,16 +49472,16 @@
     </x:row>
     <x:row r="3517">
       <x:c r="A3517" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3517" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3517" s="1" t="str">
+        <x:v>გამორთვა</x:v>
+      </x:c>
+      <x:c r="D3517" s="1" t="str">
         <x:v>выключить</x:v>
-      </x:c>
-      <x:c r="D3517" s="1" t="str">
-        <x:v>გამორთვა</x:v>
       </x:c>
     </x:row>
     <x:row r="3518">
@@ -49514,16 +49514,16 @@
     </x:row>
     <x:row r="3520">
       <x:c r="A3520" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3520" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3520" s="1" t="str">
+        <x:v>ტელეფონის ნომრით</x:v>
+      </x:c>
+      <x:c r="D3520" s="1" t="str">
         <x:v>по номеру телефона</x:v>
-      </x:c>
-      <x:c r="D3520" s="1" t="str">
-        <x:v>ტელეფონის ნომრით</x:v>
       </x:c>
     </x:row>
     <x:row r="3521">
@@ -49780,16 +49780,16 @@
     </x:row>
     <x:row r="3539">
       <x:c r="A3539" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3539" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3539" s="1" t="str">
+        <x:v>various</x:v>
+      </x:c>
+      <x:c r="D3539" s="1" t="str">
         <x:v>разнообразный</x:v>
-      </x:c>
-      <x:c r="D3539" s="1" t="str">
-        <x:v>various</x:v>
       </x:c>
     </x:row>
     <x:row r="3540">
@@ -49892,30 +49892,30 @@
     </x:row>
     <x:row r="3547">
       <x:c r="A3547" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3547" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3547" s="1" t="str">
+        <x:v>ფუნთუშები</x:v>
+      </x:c>
+      <x:c r="D3547" s="1" t="str">
         <x:v>булочки</x:v>
-      </x:c>
-      <x:c r="D3547" s="1" t="str">
-        <x:v>ფუნთუშები</x:v>
       </x:c>
     </x:row>
     <x:row r="3548">
       <x:c r="A3548" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3548" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3548" s="1" t="str">
+        <x:v>მშვენიერი</x:v>
+      </x:c>
+      <x:c r="D3548" s="1" t="str">
         <x:v>прекрасно</x:v>
-      </x:c>
-      <x:c r="D3548" s="1" t="str">
-        <x:v>მშვენიერი</x:v>
       </x:c>
     </x:row>
     <x:row r="3549">
@@ -49976,30 +49976,30 @@
     </x:row>
     <x:row r="3553">
       <x:c r="A3553" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3553" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3553" s="1" t="str">
+        <x:v>ბერძნული ენა</x:v>
+      </x:c>
+      <x:c r="D3553" s="1" t="str">
         <x:v>греческий язык</x:v>
-      </x:c>
-      <x:c r="D3553" s="1" t="str">
-        <x:v>ბერძნული ენა</x:v>
       </x:c>
     </x:row>
     <x:row r="3554">
       <x:c r="A3554" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3554" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3554" s="1" t="str">
+        <x:v>Გემრიელად მიირთვით</x:v>
+      </x:c>
+      <x:c r="D3554" s="1" t="str">
         <x:v>приятного аппетита</x:v>
-      </x:c>
-      <x:c r="D3554" s="1" t="str">
-        <x:v>Გემრიელად მიირთვით</x:v>
       </x:c>
     </x:row>
     <x:row r="3555">
@@ -50088,72 +50088,72 @@
     </x:row>
     <x:row r="3561">
       <x:c r="A3561" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3561" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3561" s="1" t="str">
+        <x:v>შეგიძლიათ აქ გაჩერდეთ</x:v>
+      </x:c>
+      <x:c r="D3561" s="1" t="str">
         <x:v>тут можно остановиться</x:v>
-      </x:c>
-      <x:c r="D3561" s="1" t="str">
-        <x:v>შეგიძლიათ აქ გაჩერდეთ</x:v>
       </x:c>
     </x:row>
     <x:row r="3562">
       <x:c r="A3562" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3562" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3562" s="1" t="str">
+        <x:v>აქ</x:v>
+      </x:c>
+      <x:c r="D3562" s="1" t="str">
         <x:v>тут</x:v>
-      </x:c>
-      <x:c r="D3562" s="1" t="str">
-        <x:v>აქ</x:v>
       </x:c>
     </x:row>
     <x:row r="3563">
       <x:c r="A3563" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3563" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3563" s="1" t="str">
+        <x:v>საბარგულში მინდა ჩავსვა</x:v>
+      </x:c>
+      <x:c r="D3563" s="1" t="str">
         <x:v>хочу положить в багажник</x:v>
-      </x:c>
-      <x:c r="D3563" s="1" t="str">
-        <x:v>საბარგულში მინდა ჩავსვა</x:v>
       </x:c>
     </x:row>
     <x:row r="3564">
       <x:c r="A3564" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3564" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3564" s="1" t="str">
+        <x:v>ძალიან გემრიელი ხორცი</x:v>
+      </x:c>
+      <x:c r="D3564" s="1" t="str">
         <x:v>очень вкусное мясо</x:v>
-      </x:c>
-      <x:c r="D3564" s="1" t="str">
-        <x:v>ძალიან გემრიელი ხორცი</x:v>
       </x:c>
     </x:row>
     <x:row r="3565">
       <x:c r="A3565" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3565" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3565" s="1" t="str">
+        <x:v>ძალიან გემრიელი მწვადი</x:v>
+      </x:c>
+      <x:c r="D3565" s="1" t="str">
         <x:v>очень вкусный шашлык</x:v>
-      </x:c>
-      <x:c r="D3565" s="1" t="str">
-        <x:v>ძალიან გემრიელი მწვადი</x:v>
       </x:c>
     </x:row>
     <x:row r="3566">
@@ -50284,58 +50284,58 @@
     </x:row>
     <x:row r="3575">
       <x:c r="A3575" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3575" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3575" s="1" t="str">
+        <x:v>დრო</x:v>
+      </x:c>
+      <x:c r="D3575" s="1" t="str">
         <x:v>время</x:v>
-      </x:c>
-      <x:c r="D3575" s="1" t="str">
-        <x:v>დრო</x:v>
       </x:c>
     </x:row>
     <x:row r="3576">
       <x:c r="A3576" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3576" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3576" s="1" t="str">
+        <x:v>მობრუნება</x:v>
+      </x:c>
+      <x:c r="D3576" s="1" t="str">
         <x:v>очередь</x:v>
-      </x:c>
-      <x:c r="D3576" s="1" t="str">
-        <x:v>მობრუნება</x:v>
       </x:c>
     </x:row>
     <x:row r="3577">
       <x:c r="A3577" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3577" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3577" s="1" t="str">
+        <x:v>ჯერჯერობით</x:v>
+      </x:c>
+      <x:c r="D3577" s="1" t="str">
         <x:v>пока всё</x:v>
-      </x:c>
-      <x:c r="D3577" s="1" t="str">
-        <x:v>ჯერჯერობით</x:v>
       </x:c>
     </x:row>
     <x:row r="3578">
       <x:c r="A3578" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3578" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3578" s="1" t="str">
+        <x:v>ყველა</x:v>
+      </x:c>
+      <x:c r="D3578" s="1" t="str">
         <x:v>всё</x:v>
-      </x:c>
-      <x:c r="D3578" s="1" t="str">
-        <x:v>ყველა</x:v>
       </x:c>
     </x:row>
     <x:row r="3579">
@@ -50466,16 +50466,16 @@
     </x:row>
     <x:row r="3588">
       <x:c r="A3588" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3588" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3588" s="1" t="str">
+        <x:v>წყალბადის ზეჟანგი</x:v>
+      </x:c>
+      <x:c r="D3588" s="1" t="str">
         <x:v>перекись водорода</x:v>
-      </x:c>
-      <x:c r="D3588" s="1" t="str">
-        <x:v>წყალბადის ზეჟანგი</x:v>
       </x:c>
     </x:row>
     <x:row r="3589">
@@ -50508,16 +50508,16 @@
     </x:row>
     <x:row r="3591">
       <x:c r="A3591" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3591" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3591" s="1" t="str">
+        <x:v>ashtray</x:v>
+      </x:c>
+      <x:c r="D3591" s="1" t="str">
         <x:v>пепельница</x:v>
-      </x:c>
-      <x:c r="D3591" s="1" t="str">
-        <x:v>ashtray</x:v>
       </x:c>
     </x:row>
     <x:row r="3592">
@@ -50536,16 +50536,16 @@
     </x:row>
     <x:row r="3593">
       <x:c r="A3593" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3593" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3593" s="1" t="str">
+        <x:v>beckon</x:v>
+      </x:c>
+      <x:c r="D3593" s="1" t="str">
         <x:v>подзывать</x:v>
-      </x:c>
-      <x:c r="D3593" s="1" t="str">
-        <x:v>beckon</x:v>
       </x:c>
     </x:row>
     <x:row r="3594">
@@ -50620,44 +50620,44 @@
     </x:row>
     <x:row r="3599">
       <x:c r="A3599" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3599" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3599" s="1" t="str">
+        <x:v>ორმოცი</x:v>
+      </x:c>
+      <x:c r="D3599" s="1" t="str">
         <x:v>сорок</x:v>
-      </x:c>
-      <x:c r="D3599" s="1" t="str">
-        <x:v>ორმოცი</x:v>
       </x:c>
     </x:row>
     <x:row r="3600">
       <x:c r="A3600" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3600" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3600" s="1" t="str">
+        <x:v>მოვიყვანე</x:v>
+      </x:c>
+      <x:c r="D3600" s="1" t="str">
         <x:v>я принес</x:v>
-      </x:c>
-      <x:c r="D3600" s="1" t="str">
-        <x:v>მოვიყვანე</x:v>
       </x:c>
     </x:row>
     <x:row r="3601">
       <x:c r="A3601" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3601" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3601" s="1" t="str">
+        <x:v>ბადრიჯანი</x:v>
+      </x:c>
+      <x:c r="D3601" s="1" t="str">
         <x:v>баклажан</x:v>
-      </x:c>
-      <x:c r="D3601" s="1" t="str">
-        <x:v>ბადრიჯანი</x:v>
       </x:c>
     </x:row>
     <x:row r="3602">
@@ -50732,44 +50732,44 @@
     </x:row>
     <x:row r="3607">
       <x:c r="A3607" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3607" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3607" s="1" t="str">
+        <x:v>კარგად არ მესმის</x:v>
+      </x:c>
+      <x:c r="D3607" s="1" t="str">
         <x:v>я плохо понимаю</x:v>
-      </x:c>
-      <x:c r="D3607" s="1" t="str">
-        <x:v>კარგად არ მესმის</x:v>
       </x:c>
     </x:row>
     <x:row r="3608">
       <x:c r="A3608" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3608" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3608" s="1" t="str">
+        <x:v>ძალიან გემრიელი</x:v>
+      </x:c>
+      <x:c r="D3608" s="1" t="str">
         <x:v>очень вкусно</x:v>
-      </x:c>
-      <x:c r="D3608" s="1" t="str">
-        <x:v>ძალიან გემრიელი</x:v>
       </x:c>
     </x:row>
     <x:row r="3609">
       <x:c r="A3609" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3609" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3609" s="1" t="str">
+        <x:v>ბოდიში მე არ მესმის</x:v>
+      </x:c>
+      <x:c r="D3609" s="1" t="str">
         <x:v>извините, я не понимаю</x:v>
-      </x:c>
-      <x:c r="D3609" s="1" t="str">
-        <x:v>ბოდიში მე არ მესმის</x:v>
       </x:c>
     </x:row>
     <x:row r="3610">
@@ -50858,30 +50858,30 @@
     </x:row>
     <x:row r="3616">
       <x:c r="A3616" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3616" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3616" s="1" t="str">
+        <x:v>buckwheat</x:v>
+      </x:c>
+      <x:c r="D3616" s="1" t="str">
         <x:v>гоечка</x:v>
-      </x:c>
-      <x:c r="D3616" s="1" t="str">
-        <x:v>buckwheat</x:v>
       </x:c>
     </x:row>
     <x:row r="3617">
       <x:c r="A3617" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3617" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3617" s="1" t="str">
+        <x:v>beet</x:v>
+      </x:c>
+      <x:c r="D3617" s="1" t="str">
         <x:v>свекла</x:v>
-      </x:c>
-      <x:c r="D3617" s="1" t="str">
-        <x:v>beet</x:v>
       </x:c>
     </x:row>
     <x:row r="3618">
@@ -51404,16 +51404,16 @@
     </x:row>
     <x:row r="3655">
       <x:c r="A3655" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3655" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3655" s="1" t="str">
+        <x:v>what new did you learn?</x:v>
+      </x:c>
+      <x:c r="D3655" s="1" t="str">
         <x:v>что нового ты узнал?</x:v>
-      </x:c>
-      <x:c r="D3655" s="1" t="str">
-        <x:v>what new did you learn?</x:v>
       </x:c>
     </x:row>
     <x:row r="3656">
@@ -52230,30 +52230,30 @@
     </x:row>
     <x:row r="3714">
       <x:c r="A3714" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3714" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3714" s="1" t="str">
+        <x:v>hatched</x:v>
+      </x:c>
+      <x:c r="D3714" s="1" t="str">
         <x:v>вылупились</x:v>
-      </x:c>
-      <x:c r="D3714" s="1" t="str">
-        <x:v>hatched</x:v>
       </x:c>
     </x:row>
     <x:row r="3715">
       <x:c r="A3715" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>English</x:v>
       </x:c>
       <x:c r="B3715" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3715" s="1" t="str">
+        <x:v>hatch</x:v>
+      </x:c>
+      <x:c r="D3715" s="1" t="str">
         <x:v>вылупляться</x:v>
-      </x:c>
-      <x:c r="D3715" s="1" t="str">
-        <x:v>hatch</x:v>
       </x:c>
     </x:row>
     <x:row r="3716">
@@ -53364,58 +53364,58 @@
     </x:row>
     <x:row r="3795">
       <x:c r="A3795" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Italian</x:v>
       </x:c>
       <x:c r="B3795" s="1" t="str">
-        <x:v>Italian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3795" s="1" t="str">
+        <x:v>guardare</x:v>
+      </x:c>
+      <x:c r="D3795" s="1" t="str">
         <x:v>смотреть</x:v>
-      </x:c>
-      <x:c r="D3795" s="1" t="str">
-        <x:v>guardare</x:v>
       </x:c>
     </x:row>
     <x:row r="3796">
       <x:c r="A3796" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Italian</x:v>
       </x:c>
       <x:c r="B3796" s="1" t="str">
-        <x:v>Italian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3796" s="1" t="str">
+        <x:v>dove?</x:v>
+      </x:c>
+      <x:c r="D3796" s="1" t="str">
         <x:v>куда?</x:v>
-      </x:c>
-      <x:c r="D3796" s="1" t="str">
-        <x:v>dove?</x:v>
       </x:c>
     </x:row>
     <x:row r="3797">
       <x:c r="A3797" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Italian</x:v>
       </x:c>
       <x:c r="B3797" s="1" t="str">
-        <x:v>Italian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3797" s="1" t="str">
+        <x:v>se</x:v>
+      </x:c>
+      <x:c r="D3797" s="1" t="str">
         <x:v>если</x:v>
-      </x:c>
-      <x:c r="D3797" s="1" t="str">
-        <x:v>se</x:v>
       </x:c>
     </x:row>
     <x:row r="3798">
       <x:c r="A3798" s="1" t="str">
-        <x:v>Russian</x:v>
+        <x:v>Italian</x:v>
       </x:c>
       <x:c r="B3798" s="1" t="str">
-        <x:v>Italian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3798" s="1" t="str">
+        <x:v>quanto</x:v>
+      </x:c>
+      <x:c r="D3798" s="1" t="str">
         <x:v>сколько</x:v>
-      </x:c>
-      <x:c r="D3798" s="1" t="str">
-        <x:v>quanto</x:v>
       </x:c>
     </x:row>
     <x:row r="3799">

</xml_diff>

<commit_message>
Enforce Russian vocabulary translations
</commit_message>
<xml_diff>
--- a/data/source/Saved translations.xlsx
+++ b/data/source/Saved translations.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saved translations" sheetId="1" r:id="R8eadaa960bcf4be1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Saved translations" sheetId="1" r:id="R79eb77d5eb834661"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -685,13 +685,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B32" s="1" t="str">
-        <x:v>German</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C32" s="1" t="str">
-        <x:v>that's so nice of you</x:v>
+        <x:v>That's so nice of you</x:v>
       </x:c>
       <x:c r="D32" s="1" t="str">
-        <x:v>Das ist sehr nett von dir.</x:v>
+        <x:v>это так мило с твоей стороны</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -1105,13 +1105,13 @@
         <x:v>German</x:v>
       </x:c>
       <x:c r="B62" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C62" s="1" t="str">
-        <x:v>Zumbeispiel</x:v>
+        <x:v>zum Beispiel</x:v>
       </x:c>
       <x:c r="D62" s="1" t="str">
-        <x:v>For example</x:v>
+        <x:v>например</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -25451,13 +25451,13 @@
         <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B1801" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C1801" s="1" t="str">
-        <x:v>აგმაშენებელი</x:v>
+        <x:v>აღმაშენებელი</x:v>
       </x:c>
       <x:c r="D1801" s="1" t="str">
-        <x:v>Builder</x:v>
+        <x:v>строитель</x:v>
       </x:c>
     </x:row>
     <x:row r="1802">
@@ -30914,7 +30914,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2191" s="1" t="str">
-        <x:v>sognia</x:v>
+        <x:v>sognava</x:v>
       </x:c>
       <x:c r="D2191" s="1" t="str">
         <x:v>он мечтал</x:v>
@@ -32017,13 +32017,13 @@
         <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B2270" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2270" s="1" t="str">
         <x:v>გულწრფელად</x:v>
       </x:c>
       <x:c r="D2270" s="1" t="str">
-        <x:v>honestly</x:v>
+        <x:v>искренне</x:v>
       </x:c>
     </x:row>
     <x:row r="2271">
@@ -33053,13 +33053,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B2344" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2344" s="1" t="str">
         <x:v>eyesight</x:v>
       </x:c>
       <x:c r="D2344" s="1" t="str">
-        <x:v>eyesight</x:v>
+        <x:v>зрение</x:v>
       </x:c>
     </x:row>
     <x:row r="2345">
@@ -35433,13 +35433,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B2514" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2514" s="1" t="str">
         <x:v>vagina</x:v>
       </x:c>
       <x:c r="D2514" s="1" t="str">
-        <x:v>საშო</x:v>
+        <x:v>влагалище</x:v>
       </x:c>
     </x:row>
     <x:row r="2515">
@@ -37435,13 +37435,13 @@
         <x:v>French</x:v>
       </x:c>
       <x:c r="B2657" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C2657" s="1" t="str">
-        <x:v>pas bies mal</x:v>
+        <x:v>pas mal</x:v>
       </x:c>
       <x:c r="D2657" s="1" t="str">
-        <x:v>not bad</x:v>
+        <x:v>неплохо</x:v>
       </x:c>
     </x:row>
     <x:row r="2658">
@@ -45166,7 +45166,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3209" s="1" t="str">
-        <x:v>შენც არ გაქვს დენი?</x:v>
+        <x:v>თქვენც არ გაქვთ დენი?</x:v>
       </x:c>
       <x:c r="D3209" s="1" t="str">
         <x:v>у вас тоже нет электричества?</x:v>
@@ -47249,13 +47249,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3358" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3358" s="1" t="str">
         <x:v>agree</x:v>
       </x:c>
       <x:c r="D3358" s="1" t="str">
-        <x:v>ვეთანხმები</x:v>
+        <x:v>соглашаться</x:v>
       </x:c>
     </x:row>
     <x:row r="3359">
@@ -47347,13 +47347,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3365" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3365" s="1" t="str">
-        <x:v>i want i cup of cold water</x:v>
+        <x:v>I want a cup of cold water</x:v>
       </x:c>
       <x:c r="D3365" s="1" t="str">
-        <x:v>მე მინდა ჭიქა ცივი წყალი</x:v>
+        <x:v>я хочу стакан холодной воды</x:v>
       </x:c>
     </x:row>
     <x:row r="3366">
@@ -47417,13 +47417,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3370" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3370" s="1" t="str">
         <x:v>name</x:v>
       </x:c>
       <x:c r="D3370" s="1" t="str">
-        <x:v>სახელი</x:v>
+        <x:v>имя</x:v>
       </x:c>
     </x:row>
     <x:row r="3371">
@@ -47504,10 +47504,10 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3376" s="1" t="str">
-        <x:v>თიკა</x:v>
+        <x:v>ჩაიდანი</x:v>
       </x:c>
       <x:c r="D3376" s="1" t="str">
-        <x:v>Чайник</x:v>
+        <x:v>чайник</x:v>
       </x:c>
     </x:row>
     <x:row r="3377">
@@ -47518,10 +47518,10 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3377" s="1" t="str">
-        <x:v>ცივი</x:v>
+        <x:v>სიცივე</x:v>
       </x:c>
       <x:c r="D3377" s="1" t="str">
-        <x:v>Холод</x:v>
+        <x:v>холод</x:v>
       </x:c>
     </x:row>
     <x:row r="3378">
@@ -48047,13 +48047,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3415" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3415" s="1" t="str">
-        <x:v>you look really cool</x:v>
+        <x:v>You look really cool</x:v>
       </x:c>
       <x:c r="D3415" s="1" t="str">
-        <x:v>მართლა მაგრად გამოიყურები</x:v>
+        <x:v>ты выглядишь очень круто</x:v>
       </x:c>
     </x:row>
     <x:row r="3416">
@@ -48061,13 +48061,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3416" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3416" s="1" t="str">
         <x:v>nice look</x:v>
       </x:c>
       <x:c r="D3416" s="1" t="str">
-        <x:v>ლამაზი გარეგნობა</x:v>
+        <x:v>классный образ</x:v>
       </x:c>
     </x:row>
     <x:row r="3417">
@@ -48176,10 +48176,10 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3424" s="1" t="str">
-        <x:v>სად არის ნაგავი?</x:v>
+        <x:v>სად არის ნაგვის ურნა?</x:v>
       </x:c>
       <x:c r="D3424" s="1" t="str">
-        <x:v>в где мусорка?</x:v>
+        <x:v>где мусорка?</x:v>
       </x:c>
     </x:row>
     <x:row r="3425">
@@ -48271,13 +48271,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3431" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3431" s="1" t="str">
-        <x:v>i cam go out here</x:v>
+        <x:v>I can go out here</x:v>
       </x:c>
       <x:c r="D3431" s="1" t="str">
-        <x:v>მე აქ გამოვედი</x:v>
+        <x:v>я могу выйти здесь</x:v>
       </x:c>
     </x:row>
     <x:row r="3432">
@@ -48285,13 +48285,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3432" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3432" s="1" t="str">
         <x:v>after</x:v>
       </x:c>
       <x:c r="D3432" s="1" t="str">
-        <x:v>შემდეგ</x:v>
+        <x:v>после</x:v>
       </x:c>
     </x:row>
     <x:row r="3433">
@@ -48299,13 +48299,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3433" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3433" s="1" t="str">
-        <x:v>may i use it</x:v>
+        <x:v>May I use it?</x:v>
       </x:c>
       <x:c r="D3433" s="1" t="str">
-        <x:v>შემიძლია გამოვიყენო</x:v>
+        <x:v>можно мне этим воспользоваться?</x:v>
       </x:c>
     </x:row>
     <x:row r="3434">
@@ -48355,13 +48355,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3437" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3437" s="1" t="str">
-        <x:v>we didn’t order this</x:v>
+        <x:v>We didn't order this</x:v>
       </x:c>
       <x:c r="D3437" s="1" t="str">
-        <x:v>ჩვენ არ შეუკვეთეთ ეს</x:v>
+        <x:v>мы это не заказывали</x:v>
       </x:c>
     </x:row>
     <x:row r="3438">
@@ -49027,13 +49027,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3485" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3485" s="1" t="str">
         <x:v>place</x:v>
       </x:c>
       <x:c r="D3485" s="1" t="str">
-        <x:v>ადგილი</x:v>
+        <x:v>место</x:v>
       </x:c>
     </x:row>
     <x:row r="3486">
@@ -49055,13 +49055,13 @@
         <x:v>Georgian</x:v>
       </x:c>
       <x:c r="B3487" s="1" t="str">
-        <x:v>English</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3487" s="1" t="str">
         <x:v>ორი ნაბიჯი</x:v>
       </x:c>
       <x:c r="D3487" s="1" t="str">
-        <x:v>two steps</x:v>
+        <x:v>два шага</x:v>
       </x:c>
     </x:row>
     <x:row r="3488">
@@ -49069,13 +49069,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3488" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3488" s="1" t="str">
         <x:v>here</x:v>
       </x:c>
       <x:c r="D3488" s="1" t="str">
-        <x:v>აქ</x:v>
+        <x:v>здесь</x:v>
       </x:c>
     </x:row>
     <x:row r="3489">
@@ -49083,13 +49083,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3489" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3489" s="1" t="str">
-        <x:v>i want to change banking set for my digital card from m to s</x:v>
+        <x:v>I want to change the banking settings for my digital card from M to S</x:v>
       </x:c>
       <x:c r="D3489" s="1" t="str">
-        <x:v>მინდა შევცვალო საბანკო ნაკრები ჩემი ციფრული ბარათისთვის m-დან s-მდე</x:v>
+        <x:v>я хочу изменить банковские настройки моей цифровой карты с M на S</x:v>
       </x:c>
     </x:row>
     <x:row r="3490">
@@ -49097,13 +49097,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3490" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3490" s="1" t="str">
-        <x:v>i want to ipen virtual card</x:v>
+        <x:v>I want to open a virtual card</x:v>
       </x:c>
       <x:c r="D3490" s="1" t="str">
-        <x:v>ვირტუალური ბარათის გახსნა მინდა</x:v>
+        <x:v>я хочу открыть виртуальную карту</x:v>
       </x:c>
     </x:row>
     <x:row r="3491">
@@ -49111,13 +49111,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3491" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3491" s="1" t="str">
-        <x:v>can you help me</x:v>
+        <x:v>Can you help me?</x:v>
       </x:c>
       <x:c r="D3491" s="1" t="str">
-        <x:v>შეგიძლიათ დამეხმაროთ</x:v>
+        <x:v>можете мне помочь?</x:v>
       </x:c>
     </x:row>
     <x:row r="3492">
@@ -49209,13 +49209,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3498" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3498" s="1" t="str">
         <x:v>street</x:v>
       </x:c>
       <x:c r="D3498" s="1" t="str">
-        <x:v>ქუჩა</x:v>
+        <x:v>улица</x:v>
       </x:c>
     </x:row>
     <x:row r="3499">
@@ -49237,13 +49237,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3500" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3500" s="1" t="str">
-        <x:v>can we quit here</x:v>
+        <x:v>Can we leave it here?</x:v>
       </x:c>
       <x:c r="D3500" s="1" t="str">
-        <x:v>შეგვიძლია აქ დავტოვოთ</x:v>
+        <x:v>можем мы оставить это здесь?</x:v>
       </x:c>
     </x:row>
     <x:row r="3501">
@@ -49282,7 +49282,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3503" s="1" t="str">
-        <x:v>ჩვენება</x:v>
+        <x:v>მაჩვენეთ</x:v>
       </x:c>
       <x:c r="D3503" s="1" t="str">
         <x:v>покажите</x:v>
@@ -49321,13 +49321,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3506" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3506" s="1" t="str">
         <x:v>nice</x:v>
       </x:c>
       <x:c r="D3506" s="1" t="str">
-        <x:v>სასიამოვნო</x:v>
+        <x:v>приятный</x:v>
       </x:c>
     </x:row>
     <x:row r="3507">
@@ -49366,7 +49366,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3509" s="1" t="str">
-        <x:v>ქათამი</x:v>
+        <x:v>ქათმის</x:v>
       </x:c>
       <x:c r="D3509" s="1" t="str">
         <x:v>куриный</x:v>
@@ -49461,13 +49461,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3516" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3516" s="1" t="str">
         <x:v>a little</x:v>
       </x:c>
       <x:c r="D3516" s="1" t="str">
-        <x:v>ცოტა</x:v>
+        <x:v>немного</x:v>
       </x:c>
     </x:row>
     <x:row r="3517">
@@ -49489,13 +49489,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3518" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3518" s="1" t="str">
-        <x:v>do you spek english</x:v>
+        <x:v>Do you speak English?</x:v>
       </x:c>
       <x:c r="D3518" s="1" t="str">
-        <x:v>ინგლისურად ლაპარაკობ</x:v>
+        <x:v>вы говорите по-английски?</x:v>
       </x:c>
     </x:row>
     <x:row r="3519">
@@ -49503,13 +49503,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3519" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3519" s="1" t="str">
         <x:v>I want to take it out</x:v>
       </x:c>
       <x:c r="D3519" s="1" t="str">
-        <x:v>მინდა გამოვიტანო</x:v>
+        <x:v>я хочу это вынести</x:v>
       </x:c>
     </x:row>
     <x:row r="3520">
@@ -49531,13 +49531,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3521" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3521" s="1" t="str">
-        <x:v>i have card</x:v>
+        <x:v>I have a card</x:v>
       </x:c>
       <x:c r="D3521" s="1" t="str">
-        <x:v>ბარათი მაქვს</x:v>
+        <x:v>у меня есть карта</x:v>
       </x:c>
     </x:row>
     <x:row r="3522">
@@ -49559,13 +49559,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3523" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3523" s="1" t="str">
-        <x:v>can you heat one croissant</x:v>
+        <x:v>Can you heat up one croissant?</x:v>
       </x:c>
       <x:c r="D3523" s="1" t="str">
-        <x:v>შეგიძლიათ ერთი კრუასანი გააცხელოთ</x:v>
+        <x:v>можете разогреть один круассан?</x:v>
       </x:c>
     </x:row>
     <x:row r="3524">
@@ -49587,13 +49587,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3525" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3525" s="1" t="str">
-        <x:v>can i pay for this tomorrow</x:v>
+        <x:v>Can I pay for this tomorrow?</x:v>
       </x:c>
       <x:c r="D3525" s="1" t="str">
-        <x:v>შემიძლია გადავიხადო ეს ხვალ</x:v>
+        <x:v>могу я заплатить за это завтра?</x:v>
       </x:c>
     </x:row>
     <x:row r="3526">
@@ -49629,13 +49629,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3528" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3528" s="1" t="str">
-        <x:v>can i take it out?</x:v>
+        <x:v>Can I take it out?</x:v>
       </x:c>
       <x:c r="D3528" s="1" t="str">
-        <x:v>შემიძლია გამოვიტანო?</x:v>
+        <x:v>могу я это вынести?</x:v>
       </x:c>
     </x:row>
     <x:row r="3529">
@@ -49643,13 +49643,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3529" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3529" s="1" t="str">
         <x:v>together</x:v>
       </x:c>
       <x:c r="D3529" s="1" t="str">
-        <x:v>ერთად</x:v>
+        <x:v>вместе</x:v>
       </x:c>
     </x:row>
     <x:row r="3530">
@@ -49657,13 +49657,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3530" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3530" s="1" t="str">
         <x:v>egg</x:v>
       </x:c>
       <x:c r="D3530" s="1" t="str">
-        <x:v>კვერცხი</x:v>
+        <x:v>яйцо</x:v>
       </x:c>
     </x:row>
     <x:row r="3531">
@@ -49685,13 +49685,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3532" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3532" s="1" t="str">
         <x:v>beer</x:v>
       </x:c>
       <x:c r="D3532" s="1" t="str">
-        <x:v>ლუდი</x:v>
+        <x:v>пиво</x:v>
       </x:c>
     </x:row>
     <x:row r="3533">
@@ -49713,13 +49713,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3534" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3534" s="1" t="str">
         <x:v>long</x:v>
       </x:c>
       <x:c r="D3534" s="1" t="str">
-        <x:v>გრძელი</x:v>
+        <x:v>длинный</x:v>
       </x:c>
     </x:row>
     <x:row r="3535">
@@ -49727,13 +49727,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3535" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3535" s="1" t="str">
         <x:v>nice music</x:v>
       </x:c>
       <x:c r="D3535" s="1" t="str">
-        <x:v>სასიამოვნო მუსიკა</x:v>
+        <x:v>приятная музыка</x:v>
       </x:c>
     </x:row>
     <x:row r="3536">
@@ -49741,13 +49741,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3536" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3536" s="1" t="str">
-        <x:v>i learn</x:v>
+        <x:v>I am learning</x:v>
       </x:c>
       <x:c r="D3536" s="1" t="str">
-        <x:v>მე ვსწავლობ</x:v>
+        <x:v>я учусь</x:v>
       </x:c>
     </x:row>
     <x:row r="3537">
@@ -49755,13 +49755,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3537" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3537" s="1" t="str">
-        <x:v>what is your name</x:v>
+        <x:v>What is your name?</x:v>
       </x:c>
       <x:c r="D3537" s="1" t="str">
-        <x:v>რა გქვია</x:v>
+        <x:v>как вас зовут?</x:v>
       </x:c>
     </x:row>
     <x:row r="3538">
@@ -49811,13 +49811,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3541" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3541" s="1" t="str">
         <x:v>tomato soup</x:v>
       </x:c>
       <x:c r="D3541" s="1" t="str">
-        <x:v>ტომატის წვნიანი</x:v>
+        <x:v>томатный суп</x:v>
       </x:c>
     </x:row>
     <x:row r="3542">
@@ -49825,13 +49825,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3542" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3542" s="1" t="str">
         <x:v>ginger</x:v>
       </x:c>
       <x:c r="D3542" s="1" t="str">
-        <x:v>ჯანჯაფილი</x:v>
+        <x:v>имбирь</x:v>
       </x:c>
     </x:row>
     <x:row r="3543">
@@ -49839,13 +49839,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3543" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3543" s="1" t="str">
-        <x:v>do you have table for three</x:v>
+        <x:v>Do you have a table for three?</x:v>
       </x:c>
       <x:c r="D3543" s="1" t="str">
-        <x:v>გაქვთ მაგიდა სამისთვის?</x:v>
+        <x:v>у вас есть столик на троих?</x:v>
       </x:c>
     </x:row>
     <x:row r="3544">
@@ -49853,13 +49853,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3544" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3544" s="1" t="str">
         <x:v>to go</x:v>
       </x:c>
       <x:c r="D3544" s="1" t="str">
-        <x:v>წასვლა</x:v>
+        <x:v>идти</x:v>
       </x:c>
     </x:row>
     <x:row r="3545">
@@ -49867,13 +49867,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3545" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3545" s="1" t="str">
         <x:v>with ham</x:v>
       </x:c>
       <x:c r="D3545" s="1" t="str">
-        <x:v>ლორით</x:v>
+        <x:v>с ветчиной</x:v>
       </x:c>
     </x:row>
     <x:row r="3546">
@@ -49912,7 +49912,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3548" s="1" t="str">
-        <x:v>მშვენიერი</x:v>
+        <x:v>მშვენივრად</x:v>
       </x:c>
       <x:c r="D3548" s="1" t="str">
         <x:v>прекрасно</x:v>
@@ -49923,13 +49923,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3549" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3549" s="1" t="str">
         <x:v>you have</x:v>
       </x:c>
       <x:c r="D3549" s="1" t="str">
-        <x:v>შენ გაქვს</x:v>
+        <x:v>у тебя есть</x:v>
       </x:c>
     </x:row>
     <x:row r="3550">
@@ -49937,13 +49937,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3550" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3550" s="1" t="str">
         <x:v>hair</x:v>
       </x:c>
       <x:c r="D3550" s="1" t="str">
-        <x:v>თმა</x:v>
+        <x:v>волосы</x:v>
       </x:c>
     </x:row>
     <x:row r="3551">
@@ -49951,13 +49951,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3551" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3551" s="1" t="str">
-        <x:v>For one trip</x:v>
+        <x:v>for one trip</x:v>
       </x:c>
       <x:c r="D3551" s="1" t="str">
-        <x:v>ერთი მოგზაურობისთვის</x:v>
+        <x:v>на одну поездку</x:v>
       </x:c>
     </x:row>
     <x:row r="3552">
@@ -49965,13 +49965,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3552" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3552" s="1" t="str">
-        <x:v>i want to withdraw my deposit money</x:v>
+        <x:v>I want to withdraw my deposit money</x:v>
       </x:c>
       <x:c r="D3552" s="1" t="str">
-        <x:v>მე მინდა გამოვიტანო ჩემი დეპოზიტის ფული</x:v>
+        <x:v>я хочу снять деньги с депозита</x:v>
       </x:c>
     </x:row>
     <x:row r="3553">
@@ -49996,7 +49996,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3554" s="1" t="str">
-        <x:v>Გემრიელად მიირთვით</x:v>
+        <x:v>გემრიელად მიირთვით</x:v>
       </x:c>
       <x:c r="D3554" s="1" t="str">
         <x:v>приятного аппетита</x:v>
@@ -50007,13 +50007,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3555" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3555" s="1" t="str">
         <x:v>this</x:v>
       </x:c>
       <x:c r="D3555" s="1" t="str">
-        <x:v>ეს</x:v>
+        <x:v>это</x:v>
       </x:c>
     </x:row>
     <x:row r="3556">
@@ -50021,13 +50021,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3556" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3556" s="1" t="str">
         <x:v>small</x:v>
       </x:c>
       <x:c r="D3556" s="1" t="str">
-        <x:v>პატარა</x:v>
+        <x:v>маленький</x:v>
       </x:c>
     </x:row>
     <x:row r="3557">
@@ -50035,13 +50035,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3557" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3557" s="1" t="str">
         <x:v>medium</x:v>
       </x:c>
       <x:c r="D3557" s="1" t="str">
-        <x:v>საშუალო</x:v>
+        <x:v>средний</x:v>
       </x:c>
     </x:row>
     <x:row r="3558">
@@ -50049,13 +50049,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3558" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3558" s="1" t="str">
         <x:v>stop</x:v>
       </x:c>
       <x:c r="D3558" s="1" t="str">
-        <x:v>გაჩერება</x:v>
+        <x:v>остановиться</x:v>
       </x:c>
     </x:row>
     <x:row r="3559">
@@ -50063,13 +50063,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3559" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3559" s="1" t="str">
         <x:v>he can</x:v>
       </x:c>
       <x:c r="D3559" s="1" t="str">
-        <x:v>მას შეუძლია</x:v>
+        <x:v>он может</x:v>
       </x:c>
     </x:row>
     <x:row r="3560">
@@ -50077,13 +50077,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3560" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3560" s="1" t="str">
         <x:v>I can</x:v>
       </x:c>
       <x:c r="D3560" s="1" t="str">
-        <x:v>მე შემიძლია</x:v>
+        <x:v>я могу</x:v>
       </x:c>
     </x:row>
     <x:row r="3561">
@@ -50161,13 +50161,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3566" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3566" s="1" t="str">
         <x:v>something like</x:v>
       </x:c>
       <x:c r="D3566" s="1" t="str">
-        <x:v>რაღაც მსგავსი</x:v>
+        <x:v>что-то вроде</x:v>
       </x:c>
     </x:row>
     <x:row r="3567">
@@ -50175,13 +50175,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3567" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3567" s="1" t="str">
-        <x:v>it was really good</x:v>
+        <x:v>It was really good</x:v>
       </x:c>
       <x:c r="D3567" s="1" t="str">
-        <x:v>მართლა კარგი იყო</x:v>
+        <x:v>это было действительно хорошо</x:v>
       </x:c>
     </x:row>
     <x:row r="3568">
@@ -50189,13 +50189,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3568" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3568" s="1" t="str">
-        <x:v>it was very delicious</x:v>
+        <x:v>It was very delicious</x:v>
       </x:c>
       <x:c r="D3568" s="1" t="str">
-        <x:v>ძალიან გემრიელი იყო</x:v>
+        <x:v>это было очень вкусно</x:v>
       </x:c>
     </x:row>
     <x:row r="3569">
@@ -50203,13 +50203,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3569" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3569" s="1" t="str">
-        <x:v>we would like to take this out</x:v>
+        <x:v>We would like to take this out</x:v>
       </x:c>
       <x:c r="D3569" s="1" t="str">
-        <x:v>ჩვენ გვინდა ამის ამოღება</x:v>
+        <x:v>мы хотели бы взять это с собой</x:v>
       </x:c>
     </x:row>
     <x:row r="3570">
@@ -50217,13 +50217,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3570" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3570" s="1" t="str">
         <x:v>breakfast</x:v>
       </x:c>
       <x:c r="D3570" s="1" t="str">
-        <x:v>საუზმე</x:v>
+        <x:v>завтрак</x:v>
       </x:c>
     </x:row>
     <x:row r="3571">
@@ -50231,13 +50231,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3571" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3571" s="1" t="str">
         <x:v>interesting</x:v>
       </x:c>
       <x:c r="D3571" s="1" t="str">
-        <x:v>საინტერესო</x:v>
+        <x:v>интересный</x:v>
       </x:c>
     </x:row>
     <x:row r="3572">
@@ -50245,13 +50245,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3572" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3572" s="1" t="str">
-        <x:v>can we order?</x:v>
+        <x:v>Can we order?</x:v>
       </x:c>
       <x:c r="D3572" s="1" t="str">
-        <x:v>შეგვიძლია შეკვეთა?</x:v>
+        <x:v>можем мы заказать?</x:v>
       </x:c>
     </x:row>
     <x:row r="3573">
@@ -50259,13 +50259,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3573" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3573" s="1" t="str">
         <x:v>pumpkin salad</x:v>
       </x:c>
       <x:c r="D3573" s="1" t="str">
-        <x:v>გოგრის სალათი</x:v>
+        <x:v>салат из тыквы</x:v>
       </x:c>
     </x:row>
     <x:row r="3574">
@@ -50273,13 +50273,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3574" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3574" s="1" t="str">
         <x:v>pumpkin</x:v>
       </x:c>
       <x:c r="D3574" s="1" t="str">
-        <x:v>გოგრა</x:v>
+        <x:v>тыква</x:v>
       </x:c>
     </x:row>
     <x:row r="3575">
@@ -50304,7 +50304,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3576" s="1" t="str">
-        <x:v>მობრუნება</x:v>
+        <x:v>რიგი</x:v>
       </x:c>
       <x:c r="D3576" s="1" t="str">
         <x:v>очередь</x:v>
@@ -50318,7 +50318,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3577" s="1" t="str">
-        <x:v>ჯერჯერობით</x:v>
+        <x:v>ჯერჯერობით სულ ესაა</x:v>
       </x:c>
       <x:c r="D3577" s="1" t="str">
         <x:v>пока всё</x:v>
@@ -50332,7 +50332,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3578" s="1" t="str">
-        <x:v>ყველა</x:v>
+        <x:v>ყველაფერი</x:v>
       </x:c>
       <x:c r="D3578" s="1" t="str">
         <x:v>всё</x:v>
@@ -50343,13 +50343,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3579" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3579" s="1" t="str">
-        <x:v>may we ask for a discount?</x:v>
+        <x:v>May we ask for a discount?</x:v>
       </x:c>
       <x:c r="D3579" s="1" t="str">
-        <x:v>შეიძლება ვითხოვოთ ფასდაკლება?</x:v>
+        <x:v>можем мы попросить скидку?</x:v>
       </x:c>
     </x:row>
     <x:row r="3580">
@@ -50357,13 +50357,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3580" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3580" s="1" t="str">
         <x:v>nice playlist</x:v>
       </x:c>
       <x:c r="D3580" s="1" t="str">
-        <x:v>ლამაზი დასაკრავი სია</x:v>
+        <x:v>хороший плейлист</x:v>
       </x:c>
     </x:row>
     <x:row r="3581">
@@ -50371,13 +50371,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3581" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3581" s="1" t="str">
         <x:v>ginger tea</x:v>
       </x:c>
       <x:c r="D3581" s="1" t="str">
-        <x:v>ჯანჯაფილის ჩაი</x:v>
+        <x:v>имбирный чай</x:v>
       </x:c>
     </x:row>
     <x:row r="3582">
@@ -50385,13 +50385,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3582" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3582" s="1" t="str">
         <x:v>move</x:v>
       </x:c>
       <x:c r="D3582" s="1" t="str">
-        <x:v>გადაადგილება</x:v>
+        <x:v>двигаться</x:v>
       </x:c>
     </x:row>
     <x:row r="3583">
@@ -50399,13 +50399,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3583" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3583" s="1" t="str">
         <x:v>go</x:v>
       </x:c>
       <x:c r="D3583" s="1" t="str">
-        <x:v>წადი</x:v>
+        <x:v>идти</x:v>
       </x:c>
     </x:row>
     <x:row r="3584">
@@ -50413,13 +50413,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3584" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3584" s="1" t="str">
-        <x:v>ery delicious</x:v>
+        <x:v>very tasty</x:v>
       </x:c>
       <x:c r="D3584" s="1" t="str">
-        <x:v>ძალიან გემრიელი</x:v>
+        <x:v>очень вкусно</x:v>
       </x:c>
     </x:row>
     <x:row r="3585">
@@ -50441,13 +50441,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3586" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3586" s="1" t="str">
-        <x:v>i would like to pay</x:v>
+        <x:v>I would like to pay</x:v>
       </x:c>
       <x:c r="D3586" s="1" t="str">
-        <x:v>მე მინდა გადავიხადო</x:v>
+        <x:v>я хотел бы заплатить</x:v>
       </x:c>
     </x:row>
     <x:row r="3587">
@@ -50640,10 +50640,10 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3600" s="1" t="str">
-        <x:v>მოვიყვანე</x:v>
+        <x:v>მოვიტანე</x:v>
       </x:c>
       <x:c r="D3600" s="1" t="str">
-        <x:v>я принес</x:v>
+        <x:v>я принёс</x:v>
       </x:c>
     </x:row>
     <x:row r="3601">
@@ -50721,13 +50721,13 @@
         <x:v>English</x:v>
       </x:c>
       <x:c r="B3606" s="1" t="str">
-        <x:v>Georgian</x:v>
+        <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3606" s="1" t="str">
         <x:v>rest</x:v>
       </x:c>
       <x:c r="D3606" s="1" t="str">
-        <x:v>დასვენება</x:v>
+        <x:v>отдыхать</x:v>
       </x:c>
     </x:row>
     <x:row r="3607">
@@ -53328,7 +53328,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3792" s="1" t="str">
-        <x:v>corta</x:v>
+        <x:v>corti</x:v>
       </x:c>
       <x:c r="D3792" s="1" t="str">
         <x:v>короткие</x:v>
@@ -53342,7 +53342,7 @@
         <x:v>Russian</x:v>
       </x:c>
       <x:c r="C3793" s="1" t="str">
-        <x:v>piu</x:v>
+        <x:v>più</x:v>
       </x:c>
       <x:c r="D3793" s="1" t="str">
         <x:v>более</x:v>

</xml_diff>